<commit_message>
cambios de firma  v2w
</commit_message>
<xml_diff>
--- a/backend-inamhi/plantillas/plantilla_ap.xlsx
+++ b/backend-inamhi/plantillas/plantilla_ap.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistemas\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistemas\Documents\inamhi rrhh\a_inamhi\backend-inamhi\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E72EE787-5315-4DDA-90FA-B4869DC33E33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{631491CE-527A-42A4-80F7-CA3C0310A4E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34785" yWindow="2580" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ap" sheetId="1" r:id="rId1"/>
@@ -1099,8 +1099,291 @@
     <xf numFmtId="37" fontId="16" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1114,21 +1397,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1148,274 +1416,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="8" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -1752,7 +1752,7 @@
           <xdr:col>9</xdr:col>
           <xdr:colOff>781050</xdr:colOff>
           <xdr:row>14</xdr:row>
-          <xdr:rowOff>38100</xdr:rowOff>
+          <xdr:rowOff>38101</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2154,7 +2154,7 @@
           <xdr:col>13</xdr:col>
           <xdr:colOff>104775</xdr:colOff>
           <xdr:row>14</xdr:row>
-          <xdr:rowOff>38100</xdr:rowOff>
+          <xdr:rowOff>38101</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2422,7 +2422,7 @@
           <xdr:col>17</xdr:col>
           <xdr:colOff>76200</xdr:colOff>
           <xdr:row>14</xdr:row>
-          <xdr:rowOff>38100</xdr:rowOff>
+          <xdr:rowOff>38101</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2690,7 +2690,7 @@
           <xdr:col>10</xdr:col>
           <xdr:colOff>742950</xdr:colOff>
           <xdr:row>21</xdr:row>
-          <xdr:rowOff>38100</xdr:rowOff>
+          <xdr:rowOff>60513</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2757,7 +2757,7 @@
           <xdr:col>12</xdr:col>
           <xdr:colOff>714375</xdr:colOff>
           <xdr:row>21</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>31938</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2824,7 +2824,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>0</xdr:colOff>
           <xdr:row>14</xdr:row>
-          <xdr:rowOff>38100</xdr:rowOff>
+          <xdr:rowOff>38101</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3579,250 +3579,250 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="95"/>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="97"/>
-      <c r="K1" s="88" t="s">
+      <c r="A1" s="141"/>
+      <c r="B1" s="142"/>
+      <c r="C1" s="142"/>
+      <c r="D1" s="142"/>
+      <c r="E1" s="142"/>
+      <c r="F1" s="142"/>
+      <c r="G1" s="142"/>
+      <c r="H1" s="142"/>
+      <c r="I1" s="142"/>
+      <c r="J1" s="143"/>
+      <c r="K1" s="136" t="s">
         <v>28</v>
       </c>
-      <c r="L1" s="89"/>
-      <c r="M1" s="89"/>
-      <c r="N1" s="89"/>
-      <c r="O1" s="89"/>
-      <c r="P1" s="89"/>
+      <c r="L1" s="137"/>
+      <c r="M1" s="137"/>
+      <c r="N1" s="137"/>
+      <c r="O1" s="137"/>
+      <c r="P1" s="137"/>
     </row>
     <row r="2" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="98"/>
-      <c r="B2" s="90"/>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="90"/>
-      <c r="H2" s="90"/>
-      <c r="I2" s="90"/>
-      <c r="J2" s="99"/>
-      <c r="K2" s="90"/>
-      <c r="L2" s="90"/>
-      <c r="M2" s="90"/>
-      <c r="N2" s="90"/>
-      <c r="O2" s="90"/>
-      <c r="P2" s="90"/>
+      <c r="A2" s="144"/>
+      <c r="B2" s="138"/>
+      <c r="C2" s="138"/>
+      <c r="D2" s="138"/>
+      <c r="E2" s="138"/>
+      <c r="F2" s="138"/>
+      <c r="G2" s="138"/>
+      <c r="H2" s="138"/>
+      <c r="I2" s="138"/>
+      <c r="J2" s="145"/>
+      <c r="K2" s="138"/>
+      <c r="L2" s="138"/>
+      <c r="M2" s="138"/>
+      <c r="N2" s="138"/>
+      <c r="O2" s="138"/>
+      <c r="P2" s="138"/>
     </row>
     <row r="3" spans="1:16" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="98"/>
-      <c r="B3" s="90"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
-      <c r="J3" s="99"/>
-      <c r="K3" s="91" t="s">
+      <c r="A3" s="144"/>
+      <c r="B3" s="138"/>
+      <c r="C3" s="138"/>
+      <c r="D3" s="138"/>
+      <c r="E3" s="138"/>
+      <c r="F3" s="138"/>
+      <c r="G3" s="138"/>
+      <c r="H3" s="138"/>
+      <c r="I3" s="138"/>
+      <c r="J3" s="145"/>
+      <c r="K3" s="94" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="92"/>
-      <c r="M3" s="119" t="s">
+      <c r="L3" s="129"/>
+      <c r="M3" s="163" t="s">
         <v>143</v>
       </c>
-      <c r="N3" s="119"/>
-      <c r="O3" s="119"/>
-      <c r="P3" s="119"/>
+      <c r="N3" s="163"/>
+      <c r="O3" s="163"/>
+      <c r="P3" s="163"/>
     </row>
     <row r="4" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="98"/>
-      <c r="B4" s="90"/>
-      <c r="C4" s="90"/>
-      <c r="D4" s="90"/>
-      <c r="E4" s="90"/>
-      <c r="F4" s="90"/>
-      <c r="G4" s="90"/>
-      <c r="H4" s="90"/>
-      <c r="I4" s="90"/>
-      <c r="J4" s="99"/>
-      <c r="K4" s="91" t="s">
+      <c r="A4" s="144"/>
+      <c r="B4" s="138"/>
+      <c r="C4" s="138"/>
+      <c r="D4" s="138"/>
+      <c r="E4" s="138"/>
+      <c r="F4" s="138"/>
+      <c r="G4" s="138"/>
+      <c r="H4" s="138"/>
+      <c r="I4" s="138"/>
+      <c r="J4" s="145"/>
+      <c r="K4" s="94" t="s">
         <v>30</v>
       </c>
-      <c r="L4" s="92"/>
-      <c r="M4" s="92"/>
-      <c r="N4" s="92"/>
-      <c r="O4" s="92"/>
-      <c r="P4" s="92"/>
+      <c r="L4" s="129"/>
+      <c r="M4" s="129"/>
+      <c r="N4" s="129"/>
+      <c r="O4" s="129"/>
+      <c r="P4" s="129"/>
     </row>
     <row r="5" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="100"/>
-      <c r="B5" s="101"/>
-      <c r="C5" s="101"/>
-      <c r="D5" s="101"/>
-      <c r="E5" s="101"/>
-      <c r="F5" s="101"/>
-      <c r="G5" s="101"/>
-      <c r="H5" s="101"/>
-      <c r="I5" s="101"/>
-      <c r="J5" s="102"/>
-      <c r="K5" s="93">
+      <c r="A5" s="146"/>
+      <c r="B5" s="147"/>
+      <c r="C5" s="147"/>
+      <c r="D5" s="147"/>
+      <c r="E5" s="147"/>
+      <c r="F5" s="147"/>
+      <c r="G5" s="147"/>
+      <c r="H5" s="147"/>
+      <c r="I5" s="147"/>
+      <c r="J5" s="148"/>
+      <c r="K5" s="139">
         <v>46121</v>
       </c>
-      <c r="L5" s="94"/>
-      <c r="M5" s="94"/>
-      <c r="N5" s="94"/>
-      <c r="O5" s="94"/>
-      <c r="P5" s="94"/>
+      <c r="L5" s="140"/>
+      <c r="M5" s="140"/>
+      <c r="N5" s="140"/>
+      <c r="O5" s="140"/>
+      <c r="P5" s="140"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="120"/>
-      <c r="B6" s="109"/>
-      <c r="C6" s="109"/>
-      <c r="D6" s="109"/>
-      <c r="E6" s="109"/>
-      <c r="F6" s="109"/>
-      <c r="G6" s="109"/>
-      <c r="H6" s="110"/>
-      <c r="I6" s="109"/>
-      <c r="J6" s="109"/>
-      <c r="K6" s="109"/>
-      <c r="L6" s="109"/>
-      <c r="M6" s="109"/>
-      <c r="N6" s="109"/>
-      <c r="O6" s="109"/>
-      <c r="P6" s="110"/>
+      <c r="A6" s="164"/>
+      <c r="B6" s="155"/>
+      <c r="C6" s="155"/>
+      <c r="D6" s="155"/>
+      <c r="E6" s="155"/>
+      <c r="F6" s="155"/>
+      <c r="G6" s="155"/>
+      <c r="H6" s="156"/>
+      <c r="I6" s="155"/>
+      <c r="J6" s="155"/>
+      <c r="K6" s="155"/>
+      <c r="L6" s="155"/>
+      <c r="M6" s="155"/>
+      <c r="N6" s="155"/>
+      <c r="O6" s="155"/>
+      <c r="P6" s="156"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="121"/>
-      <c r="B7" s="111"/>
-      <c r="C7" s="111"/>
-      <c r="D7" s="111"/>
-      <c r="E7" s="111"/>
-      <c r="F7" s="111"/>
-      <c r="G7" s="111"/>
-      <c r="H7" s="112"/>
-      <c r="I7" s="111"/>
-      <c r="J7" s="111"/>
-      <c r="K7" s="111"/>
-      <c r="L7" s="111"/>
-      <c r="M7" s="111"/>
-      <c r="N7" s="111"/>
-      <c r="O7" s="111"/>
-      <c r="P7" s="112"/>
+      <c r="A7" s="165"/>
+      <c r="B7" s="157"/>
+      <c r="C7" s="157"/>
+      <c r="D7" s="157"/>
+      <c r="E7" s="157"/>
+      <c r="F7" s="157"/>
+      <c r="G7" s="157"/>
+      <c r="H7" s="158"/>
+      <c r="I7" s="157"/>
+      <c r="J7" s="157"/>
+      <c r="K7" s="157"/>
+      <c r="L7" s="157"/>
+      <c r="M7" s="157"/>
+      <c r="N7" s="157"/>
+      <c r="O7" s="157"/>
+      <c r="P7" s="158"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="122" t="s">
+      <c r="A8" s="166" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="113"/>
-      <c r="C8" s="113"/>
-      <c r="D8" s="113"/>
-      <c r="E8" s="113"/>
-      <c r="F8" s="113"/>
-      <c r="G8" s="113"/>
-      <c r="H8" s="114"/>
-      <c r="I8" s="113" t="s">
+      <c r="B8" s="159"/>
+      <c r="C8" s="159"/>
+      <c r="D8" s="159"/>
+      <c r="E8" s="159"/>
+      <c r="F8" s="159"/>
+      <c r="G8" s="159"/>
+      <c r="H8" s="160"/>
+      <c r="I8" s="159" t="s">
         <v>2</v>
       </c>
-      <c r="J8" s="113"/>
-      <c r="K8" s="113"/>
-      <c r="L8" s="113"/>
-      <c r="M8" s="113"/>
-      <c r="N8" s="113"/>
-      <c r="O8" s="113"/>
-      <c r="P8" s="114"/>
+      <c r="J8" s="159"/>
+      <c r="K8" s="159"/>
+      <c r="L8" s="159"/>
+      <c r="M8" s="159"/>
+      <c r="N8" s="159"/>
+      <c r="O8" s="159"/>
+      <c r="P8" s="160"/>
     </row>
     <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="103" t="s">
+      <c r="A9" s="149" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="104"/>
-      <c r="C9" s="104"/>
-      <c r="D9" s="105"/>
-      <c r="E9" s="103" t="s">
+      <c r="B9" s="150"/>
+      <c r="C9" s="150"/>
+      <c r="D9" s="151"/>
+      <c r="E9" s="149" t="s">
         <v>48</v>
       </c>
-      <c r="F9" s="104"/>
-      <c r="G9" s="104"/>
-      <c r="H9" s="105"/>
-      <c r="I9" s="91" t="s">
+      <c r="F9" s="150"/>
+      <c r="G9" s="150"/>
+      <c r="H9" s="151"/>
+      <c r="I9" s="94" t="s">
         <v>29</v>
       </c>
-      <c r="J9" s="92"/>
-      <c r="K9" s="92"/>
-      <c r="L9" s="92"/>
-      <c r="M9" s="92"/>
-      <c r="N9" s="92"/>
-      <c r="O9" s="92"/>
-      <c r="P9" s="92"/>
+      <c r="J9" s="129"/>
+      <c r="K9" s="129"/>
+      <c r="L9" s="129"/>
+      <c r="M9" s="129"/>
+      <c r="N9" s="129"/>
+      <c r="O9" s="129"/>
+      <c r="P9" s="129"/>
     </row>
     <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="106"/>
-      <c r="B10" s="107"/>
-      <c r="C10" s="107"/>
-      <c r="D10" s="108"/>
-      <c r="E10" s="106"/>
-      <c r="F10" s="107"/>
-      <c r="G10" s="107"/>
-      <c r="H10" s="108"/>
-      <c r="I10" s="115" t="s">
+      <c r="A10" s="152"/>
+      <c r="B10" s="153"/>
+      <c r="C10" s="153"/>
+      <c r="D10" s="154"/>
+      <c r="E10" s="152"/>
+      <c r="F10" s="153"/>
+      <c r="G10" s="153"/>
+      <c r="H10" s="154"/>
+      <c r="I10" s="92" t="s">
         <v>42</v>
       </c>
-      <c r="J10" s="116"/>
-      <c r="K10" s="116"/>
-      <c r="L10" s="91"/>
-      <c r="M10" s="115" t="s">
+      <c r="J10" s="93"/>
+      <c r="K10" s="93"/>
+      <c r="L10" s="94"/>
+      <c r="M10" s="92" t="s">
         <v>131</v>
       </c>
-      <c r="N10" s="116"/>
-      <c r="O10" s="116"/>
-      <c r="P10" s="91"/>
+      <c r="N10" s="93"/>
+      <c r="O10" s="93"/>
+      <c r="P10" s="94"/>
     </row>
     <row r="11" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="70" t="s">
+      <c r="A11" s="167" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="71"/>
-      <c r="C11" s="71"/>
-      <c r="D11" s="71"/>
-      <c r="E11" s="70"/>
-      <c r="F11" s="71"/>
-      <c r="G11" s="71"/>
-      <c r="H11" s="72"/>
-      <c r="I11" s="78"/>
-      <c r="J11" s="79"/>
-      <c r="K11" s="79"/>
-      <c r="L11" s="80"/>
-      <c r="M11" s="78"/>
-      <c r="N11" s="79"/>
-      <c r="O11" s="79"/>
-      <c r="P11" s="80"/>
+      <c r="B11" s="168"/>
+      <c r="C11" s="168"/>
+      <c r="D11" s="168"/>
+      <c r="E11" s="167"/>
+      <c r="F11" s="168"/>
+      <c r="G11" s="168"/>
+      <c r="H11" s="169"/>
+      <c r="I11" s="170"/>
+      <c r="J11" s="171"/>
+      <c r="K11" s="171"/>
+      <c r="L11" s="172"/>
+      <c r="M11" s="170"/>
+      <c r="N11" s="171"/>
+      <c r="O11" s="171"/>
+      <c r="P11" s="172"/>
     </row>
     <row r="12" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="81" t="s">
+      <c r="A12" s="173" t="s">
         <v>132</v>
       </c>
-      <c r="B12" s="82"/>
-      <c r="C12" s="82"/>
-      <c r="D12" s="82"/>
-      <c r="E12" s="82"/>
-      <c r="F12" s="82"/>
-      <c r="G12" s="82"/>
-      <c r="H12" s="82"/>
-      <c r="I12" s="82"/>
-      <c r="J12" s="82"/>
-      <c r="K12" s="82"/>
-      <c r="L12" s="82"/>
-      <c r="M12" s="82"/>
-      <c r="N12" s="82"/>
-      <c r="O12" s="82"/>
-      <c r="P12" s="83"/>
-    </row>
-    <row r="13" spans="1:16" ht="9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="174"/>
+      <c r="C12" s="174"/>
+      <c r="D12" s="174"/>
+      <c r="E12" s="174"/>
+      <c r="F12" s="174"/>
+      <c r="G12" s="174"/>
+      <c r="H12" s="174"/>
+      <c r="I12" s="174"/>
+      <c r="J12" s="174"/>
+      <c r="K12" s="174"/>
+      <c r="L12" s="174"/>
+      <c r="M12" s="174"/>
+      <c r="N12" s="174"/>
+      <c r="O12" s="174"/>
+      <c r="P12" s="175"/>
+    </row>
+    <row r="13" spans="1:16" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -3859,19 +3859,19 @@
       </c>
       <c r="K14" s="23"/>
       <c r="L14" s="23"/>
-      <c r="M14" s="84" t="s">
+      <c r="M14" s="176" t="s">
         <v>15</v>
       </c>
-      <c r="N14" s="84"/>
-      <c r="O14" s="84"/>
+      <c r="N14" s="176"/>
+      <c r="O14" s="176"/>
       <c r="P14" s="2"/>
     </row>
     <row r="15" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="6"/>
-      <c r="B15" s="87" t="s">
+      <c r="B15" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="87"/>
+      <c r="C15" s="78"/>
       <c r="D15" s="38"/>
       <c r="E15" s="23" t="s">
         <v>9</v>
@@ -3885,19 +3885,19 @@
       </c>
       <c r="K15" s="23"/>
       <c r="L15" s="23"/>
-      <c r="M15" s="84" t="s">
+      <c r="M15" s="176" t="s">
         <v>56</v>
       </c>
-      <c r="N15" s="84"/>
-      <c r="O15" s="84"/>
+      <c r="N15" s="176"/>
+      <c r="O15" s="176"/>
       <c r="P15" s="2"/>
     </row>
     <row r="16" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
-      <c r="B16" s="87" t="s">
+      <c r="B16" s="78" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="87"/>
+      <c r="C16" s="78"/>
       <c r="D16" s="38"/>
       <c r="E16" s="23" t="s">
         <v>21</v>
@@ -3911,17 +3911,17 @@
       </c>
       <c r="K16" s="23"/>
       <c r="L16" s="23"/>
-      <c r="M16" s="85"/>
-      <c r="N16" s="85"/>
-      <c r="O16" s="85"/>
+      <c r="M16" s="162"/>
+      <c r="N16" s="162"/>
+      <c r="O16" s="162"/>
       <c r="P16" s="2"/>
     </row>
     <row r="17" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="6"/>
-      <c r="B17" s="87" t="s">
+      <c r="B17" s="78" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="87"/>
+      <c r="C17" s="78"/>
       <c r="D17" s="38"/>
       <c r="E17" s="23" t="s">
         <v>10</v>
@@ -3935,17 +3935,17 @@
       </c>
       <c r="K17" s="23"/>
       <c r="L17" s="23"/>
-      <c r="M17" s="86"/>
-      <c r="N17" s="86"/>
-      <c r="O17" s="86"/>
+      <c r="M17" s="161"/>
+      <c r="N17" s="161"/>
+      <c r="O17" s="161"/>
       <c r="P17" s="2"/>
     </row>
     <row r="18" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="6"/>
-      <c r="B18" s="87" t="s">
+      <c r="B18" s="78" t="s">
         <v>4</v>
       </c>
-      <c r="C18" s="87"/>
+      <c r="C18" s="78"/>
       <c r="D18" s="38"/>
       <c r="E18" s="23" t="s">
         <v>22</v>
@@ -3959,17 +3959,17 @@
       </c>
       <c r="K18" s="23"/>
       <c r="L18" s="23"/>
-      <c r="M18" s="146"/>
-      <c r="N18" s="146"/>
-      <c r="O18" s="146"/>
+      <c r="M18" s="105"/>
+      <c r="N18" s="105"/>
+      <c r="O18" s="105"/>
       <c r="P18" s="2"/>
     </row>
     <row r="19" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="6"/>
-      <c r="B19" s="87" t="s">
+      <c r="B19" s="78" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="87"/>
+      <c r="C19" s="78"/>
       <c r="D19" s="38"/>
       <c r="E19" s="23" t="s">
         <v>23</v>
@@ -3983,52 +3983,52 @@
       </c>
       <c r="K19" s="23"/>
       <c r="L19" s="23"/>
-      <c r="M19" s="86"/>
-      <c r="N19" s="86"/>
-      <c r="O19" s="86"/>
+      <c r="M19" s="161"/>
+      <c r="N19" s="161"/>
+      <c r="O19" s="161"/>
       <c r="P19" s="2"/>
     </row>
-    <row r="20" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6"/>
-      <c r="B20" s="77" t="s">
+      <c r="B20" s="124" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="77"/>
-      <c r="D20" s="77"/>
-      <c r="E20" s="77"/>
-      <c r="F20" s="77"/>
-      <c r="G20" s="145"/>
-      <c r="H20" s="145"/>
-      <c r="I20" s="145"/>
-      <c r="J20" s="145"/>
-      <c r="K20" s="145"/>
-      <c r="L20" s="145"/>
-      <c r="M20" s="145"/>
-      <c r="N20" s="145"/>
-      <c r="O20" s="145"/>
+      <c r="C20" s="124"/>
+      <c r="D20" s="124"/>
+      <c r="E20" s="124"/>
+      <c r="F20" s="124"/>
+      <c r="G20" s="104"/>
+      <c r="H20" s="104"/>
+      <c r="I20" s="104"/>
+      <c r="J20" s="104"/>
+      <c r="K20" s="104"/>
+      <c r="L20" s="104"/>
+      <c r="M20" s="104"/>
+      <c r="N20" s="104"/>
+      <c r="O20" s="104"/>
       <c r="P20" s="2"/>
     </row>
-    <row r="21" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6"/>
-      <c r="B21" s="153" t="s">
+      <c r="B21" s="79" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="153"/>
-      <c r="D21" s="153"/>
-      <c r="E21" s="153"/>
-      <c r="F21" s="153"/>
-      <c r="G21" s="153"/>
-      <c r="H21" s="153"/>
-      <c r="I21" s="153"/>
-      <c r="J21" s="153"/>
-      <c r="K21" s="153"/>
-      <c r="L21" s="153"/>
-      <c r="M21" s="154"/>
-      <c r="N21" s="154"/>
-      <c r="O21" s="154"/>
+      <c r="C21" s="79"/>
+      <c r="D21" s="79"/>
+      <c r="E21" s="79"/>
+      <c r="F21" s="79"/>
+      <c r="G21" s="79"/>
+      <c r="H21" s="79"/>
+      <c r="I21" s="79"/>
+      <c r="J21" s="79"/>
+      <c r="K21" s="79"/>
+      <c r="L21" s="79"/>
+      <c r="M21" s="80"/>
+      <c r="N21" s="80"/>
+      <c r="O21" s="80"/>
       <c r="P21" s="2"/>
     </row>
-    <row r="22" spans="1:16" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10"/>
       <c r="B22" s="11"/>
       <c r="C22" s="11"/>
@@ -4041,74 +4041,74 @@
       <c r="J22" s="11"/>
       <c r="K22" s="11"/>
       <c r="L22" s="11"/>
-      <c r="M22" s="85"/>
-      <c r="N22" s="85"/>
-      <c r="O22" s="85"/>
+      <c r="M22" s="162"/>
+      <c r="N22" s="162"/>
+      <c r="O22" s="162"/>
       <c r="P22" s="3"/>
     </row>
     <row r="23" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="139" t="s">
+      <c r="A23" s="116" t="s">
         <v>84</v>
       </c>
-      <c r="B23" s="140"/>
-      <c r="C23" s="140"/>
-      <c r="D23" s="140"/>
-      <c r="E23" s="140"/>
-      <c r="F23" s="140"/>
-      <c r="G23" s="140"/>
-      <c r="H23" s="140"/>
-      <c r="I23" s="140"/>
-      <c r="J23" s="140"/>
-      <c r="K23" s="140"/>
-      <c r="L23" s="140"/>
-      <c r="M23" s="140"/>
-      <c r="N23" s="140"/>
-      <c r="O23" s="140"/>
-      <c r="P23" s="141"/>
-    </row>
-    <row r="24" spans="1:16" ht="126" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="149" t="s">
+      <c r="B23" s="117"/>
+      <c r="C23" s="117"/>
+      <c r="D23" s="117"/>
+      <c r="E23" s="117"/>
+      <c r="F23" s="117"/>
+      <c r="G23" s="117"/>
+      <c r="H23" s="117"/>
+      <c r="I23" s="117"/>
+      <c r="J23" s="117"/>
+      <c r="K23" s="117"/>
+      <c r="L23" s="117"/>
+      <c r="M23" s="117"/>
+      <c r="N23" s="117"/>
+      <c r="O23" s="117"/>
+      <c r="P23" s="118"/>
+    </row>
+    <row r="24" spans="1:16" ht="116.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="109" t="s">
         <v>144</v>
       </c>
-      <c r="B24" s="150"/>
-      <c r="C24" s="150"/>
-      <c r="D24" s="150"/>
-      <c r="E24" s="150"/>
-      <c r="F24" s="150"/>
-      <c r="G24" s="150"/>
-      <c r="H24" s="150"/>
-      <c r="I24" s="150"/>
-      <c r="J24" s="150"/>
-      <c r="K24" s="150"/>
-      <c r="L24" s="150"/>
-      <c r="M24" s="150"/>
-      <c r="N24" s="150"/>
-      <c r="O24" s="150"/>
+      <c r="B24" s="110"/>
+      <c r="C24" s="110"/>
+      <c r="D24" s="110"/>
+      <c r="E24" s="110"/>
+      <c r="F24" s="110"/>
+      <c r="G24" s="110"/>
+      <c r="H24" s="110"/>
+      <c r="I24" s="110"/>
+      <c r="J24" s="110"/>
+      <c r="K24" s="110"/>
+      <c r="L24" s="110"/>
+      <c r="M24" s="110"/>
+      <c r="N24" s="110"/>
+      <c r="O24" s="110"/>
       <c r="P24" s="39"/>
     </row>
     <row r="25" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="115" t="s">
+      <c r="A25" s="92" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="116"/>
-      <c r="C25" s="116"/>
-      <c r="D25" s="116"/>
-      <c r="E25" s="116"/>
-      <c r="F25" s="116"/>
-      <c r="G25" s="116"/>
-      <c r="H25" s="91"/>
-      <c r="I25" s="115" t="s">
+      <c r="B25" s="93"/>
+      <c r="C25" s="93"/>
+      <c r="D25" s="93"/>
+      <c r="E25" s="93"/>
+      <c r="F25" s="93"/>
+      <c r="G25" s="93"/>
+      <c r="H25" s="94"/>
+      <c r="I25" s="92" t="s">
         <v>13</v>
       </c>
-      <c r="J25" s="116"/>
-      <c r="K25" s="116"/>
-      <c r="L25" s="116"/>
-      <c r="M25" s="116"/>
-      <c r="N25" s="116"/>
-      <c r="O25" s="116"/>
-      <c r="P25" s="91"/>
-    </row>
-    <row r="26" spans="1:16" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J25" s="93"/>
+      <c r="K25" s="93"/>
+      <c r="L25" s="93"/>
+      <c r="M25" s="93"/>
+      <c r="N25" s="93"/>
+      <c r="O25" s="93"/>
+      <c r="P25" s="94"/>
+    </row>
+    <row r="26" spans="1:16" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="24"/>
       <c r="B26" s="24"/>
       <c r="C26" s="24"/>
@@ -4127,269 +4127,269 @@
       <c r="P26" s="24"/>
     </row>
     <row r="27" spans="1:16" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="117" t="s">
+      <c r="A27" s="113" t="s">
         <v>72</v>
       </c>
-      <c r="B27" s="118"/>
-      <c r="C27" s="118"/>
-      <c r="D27" s="118"/>
-      <c r="E27" s="118"/>
-      <c r="F27" s="118"/>
-      <c r="G27" s="118"/>
+      <c r="B27" s="114"/>
+      <c r="C27" s="114"/>
+      <c r="D27" s="114"/>
+      <c r="E27" s="114"/>
+      <c r="F27" s="114"/>
+      <c r="G27" s="114"/>
       <c r="H27" s="65"/>
-      <c r="I27" s="117" t="s">
+      <c r="I27" s="113" t="s">
         <v>72</v>
       </c>
-      <c r="J27" s="118"/>
-      <c r="K27" s="118"/>
-      <c r="L27" s="118"/>
-      <c r="M27" s="118"/>
-      <c r="N27" s="118"/>
-      <c r="O27" s="118"/>
-      <c r="P27" s="152"/>
+      <c r="J27" s="114"/>
+      <c r="K27" s="114"/>
+      <c r="L27" s="114"/>
+      <c r="M27" s="114"/>
+      <c r="N27" s="114"/>
+      <c r="O27" s="114"/>
+      <c r="P27" s="115"/>
     </row>
     <row r="28" spans="1:16" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="13"/>
-      <c r="B28" s="75" t="s">
+      <c r="B28" s="103" t="s">
         <v>76</v>
       </c>
-      <c r="C28" s="75"/>
-      <c r="D28" s="75"/>
-      <c r="E28" s="75"/>
-      <c r="F28" s="75"/>
-      <c r="G28" s="75"/>
+      <c r="C28" s="103"/>
+      <c r="D28" s="103"/>
+      <c r="E28" s="103"/>
+      <c r="F28" s="103"/>
+      <c r="G28" s="103"/>
       <c r="H28" s="43"/>
       <c r="I28" s="13"/>
-      <c r="J28" s="75" t="s">
+      <c r="J28" s="103" t="s">
         <v>85</v>
       </c>
-      <c r="K28" s="75"/>
-      <c r="L28" s="75"/>
-      <c r="M28" s="75"/>
-      <c r="N28" s="75"/>
-      <c r="O28" s="75"/>
+      <c r="K28" s="103"/>
+      <c r="L28" s="103"/>
+      <c r="M28" s="103"/>
+      <c r="N28" s="103"/>
+      <c r="O28" s="103"/>
       <c r="P28" s="12"/>
     </row>
     <row r="29" spans="1:16" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="73" t="s">
+      <c r="A29" s="100" t="s">
         <v>77</v>
       </c>
-      <c r="B29" s="74"/>
-      <c r="C29" s="74"/>
-      <c r="D29" s="74"/>
-      <c r="E29" s="74"/>
-      <c r="F29" s="74"/>
-      <c r="G29" s="74"/>
+      <c r="B29" s="101"/>
+      <c r="C29" s="101"/>
+      <c r="D29" s="101"/>
+      <c r="E29" s="101"/>
+      <c r="F29" s="101"/>
+      <c r="G29" s="101"/>
       <c r="H29" s="66"/>
-      <c r="I29" s="73" t="s">
+      <c r="I29" s="100" t="s">
         <v>73</v>
       </c>
-      <c r="J29" s="74"/>
-      <c r="K29" s="74"/>
-      <c r="L29" s="74"/>
-      <c r="M29" s="74"/>
-      <c r="N29" s="74"/>
-      <c r="O29" s="74"/>
-      <c r="P29" s="76"/>
+      <c r="J29" s="101"/>
+      <c r="K29" s="101"/>
+      <c r="L29" s="101"/>
+      <c r="M29" s="101"/>
+      <c r="N29" s="101"/>
+      <c r="O29" s="101"/>
+      <c r="P29" s="102"/>
     </row>
     <row r="30" spans="1:16" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="13"/>
-      <c r="B30" s="75"/>
-      <c r="C30" s="75"/>
-      <c r="D30" s="75"/>
-      <c r="E30" s="75"/>
-      <c r="F30" s="75"/>
-      <c r="G30" s="75"/>
+      <c r="B30" s="103"/>
+      <c r="C30" s="103"/>
+      <c r="D30" s="103"/>
+      <c r="E30" s="103"/>
+      <c r="F30" s="103"/>
+      <c r="G30" s="103"/>
       <c r="H30" s="43"/>
       <c r="I30" s="13"/>
-      <c r="J30" s="75" t="s">
+      <c r="J30" s="103" t="s">
         <v>78</v>
       </c>
-      <c r="K30" s="75"/>
-      <c r="L30" s="75"/>
-      <c r="M30" s="75"/>
-      <c r="N30" s="75"/>
-      <c r="O30" s="75"/>
+      <c r="K30" s="103"/>
+      <c r="L30" s="103"/>
+      <c r="M30" s="103"/>
+      <c r="N30" s="103"/>
+      <c r="O30" s="103"/>
       <c r="P30" s="12"/>
     </row>
     <row r="31" spans="1:16" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="73" t="s">
+      <c r="A31" s="100" t="s">
         <v>133</v>
       </c>
-      <c r="B31" s="74"/>
-      <c r="C31" s="74"/>
-      <c r="D31" s="74"/>
-      <c r="E31" s="74"/>
-      <c r="F31" s="74"/>
-      <c r="G31" s="74"/>
+      <c r="B31" s="101"/>
+      <c r="C31" s="101"/>
+      <c r="D31" s="101"/>
+      <c r="E31" s="101"/>
+      <c r="F31" s="101"/>
+      <c r="G31" s="101"/>
       <c r="H31" s="66"/>
-      <c r="I31" s="73" t="s">
+      <c r="I31" s="100" t="s">
         <v>74</v>
       </c>
-      <c r="J31" s="74"/>
-      <c r="K31" s="74"/>
-      <c r="L31" s="74"/>
-      <c r="M31" s="74"/>
-      <c r="N31" s="74"/>
-      <c r="O31" s="74"/>
-      <c r="P31" s="76"/>
+      <c r="J31" s="101"/>
+      <c r="K31" s="101"/>
+      <c r="L31" s="101"/>
+      <c r="M31" s="101"/>
+      <c r="N31" s="101"/>
+      <c r="O31" s="101"/>
+      <c r="P31" s="102"/>
     </row>
     <row r="32" spans="1:16" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="13"/>
-      <c r="B32" s="75" t="s">
+      <c r="B32" s="103" t="s">
         <v>94</v>
       </c>
-      <c r="C32" s="75"/>
-      <c r="D32" s="75"/>
-      <c r="E32" s="75"/>
-      <c r="F32" s="75"/>
-      <c r="G32" s="75"/>
+      <c r="C32" s="103"/>
+      <c r="D32" s="103"/>
+      <c r="E32" s="103"/>
+      <c r="F32" s="103"/>
+      <c r="G32" s="103"/>
       <c r="H32" s="67"/>
       <c r="I32" s="13"/>
-      <c r="J32" s="75" t="s">
+      <c r="J32" s="103" t="s">
         <v>95</v>
       </c>
-      <c r="K32" s="75"/>
-      <c r="L32" s="75"/>
-      <c r="M32" s="75"/>
-      <c r="N32" s="75"/>
-      <c r="O32" s="75"/>
+      <c r="K32" s="103"/>
+      <c r="L32" s="103"/>
+      <c r="M32" s="103"/>
+      <c r="N32" s="103"/>
+      <c r="O32" s="103"/>
       <c r="P32" s="12"/>
     </row>
     <row r="33" spans="1:22" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="73" t="s">
+      <c r="A33" s="100" t="s">
         <v>75</v>
       </c>
-      <c r="B33" s="74"/>
-      <c r="C33" s="74"/>
-      <c r="D33" s="74"/>
-      <c r="E33" s="74"/>
-      <c r="F33" s="74"/>
-      <c r="G33" s="74"/>
+      <c r="B33" s="101"/>
+      <c r="C33" s="101"/>
+      <c r="D33" s="101"/>
+      <c r="E33" s="101"/>
+      <c r="F33" s="101"/>
+      <c r="G33" s="101"/>
       <c r="H33" s="66"/>
-      <c r="I33" s="73" t="s">
+      <c r="I33" s="100" t="s">
         <v>75</v>
       </c>
-      <c r="J33" s="74"/>
-      <c r="K33" s="74"/>
-      <c r="L33" s="74"/>
-      <c r="M33" s="74"/>
-      <c r="N33" s="74"/>
-      <c r="O33" s="74"/>
-      <c r="P33" s="76"/>
+      <c r="J33" s="101"/>
+      <c r="K33" s="101"/>
+      <c r="L33" s="101"/>
+      <c r="M33" s="101"/>
+      <c r="N33" s="101"/>
+      <c r="O33" s="101"/>
+      <c r="P33" s="102"/>
     </row>
     <row r="34" spans="1:22" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="13"/>
-      <c r="B34" s="75" t="s">
+      <c r="B34" s="103" t="s">
         <v>80</v>
       </c>
-      <c r="C34" s="75"/>
-      <c r="D34" s="75"/>
-      <c r="E34" s="75"/>
-      <c r="F34" s="75"/>
-      <c r="G34" s="75"/>
+      <c r="C34" s="103"/>
+      <c r="D34" s="103"/>
+      <c r="E34" s="103"/>
+      <c r="F34" s="103"/>
+      <c r="G34" s="103"/>
       <c r="H34" s="67"/>
       <c r="I34" s="13"/>
-      <c r="J34" s="75" t="s">
+      <c r="J34" s="103" t="s">
         <v>80</v>
       </c>
-      <c r="K34" s="75"/>
-      <c r="L34" s="75"/>
-      <c r="M34" s="75"/>
-      <c r="N34" s="75"/>
-      <c r="O34" s="75"/>
+      <c r="K34" s="103"/>
+      <c r="L34" s="103"/>
+      <c r="M34" s="103"/>
+      <c r="N34" s="103"/>
+      <c r="O34" s="103"/>
       <c r="P34" s="12"/>
     </row>
     <row r="35" spans="1:22" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="137" t="s">
+      <c r="A35" s="125" t="s">
         <v>31</v>
       </c>
-      <c r="B35" s="138"/>
-      <c r="C35" s="138"/>
-      <c r="D35" s="138"/>
-      <c r="E35" s="138"/>
-      <c r="F35" s="138"/>
-      <c r="G35" s="138"/>
+      <c r="B35" s="126"/>
+      <c r="C35" s="126"/>
+      <c r="D35" s="126"/>
+      <c r="E35" s="126"/>
+      <c r="F35" s="126"/>
+      <c r="G35" s="126"/>
       <c r="H35" s="66"/>
-      <c r="I35" s="73" t="s">
+      <c r="I35" s="100" t="s">
         <v>31</v>
       </c>
-      <c r="J35" s="74"/>
-      <c r="K35" s="74"/>
-      <c r="L35" s="74"/>
-      <c r="M35" s="74"/>
-      <c r="N35" s="74"/>
-      <c r="O35" s="74"/>
-      <c r="P35" s="76"/>
+      <c r="J35" s="101"/>
+      <c r="K35" s="101"/>
+      <c r="L35" s="101"/>
+      <c r="M35" s="101"/>
+      <c r="N35" s="101"/>
+      <c r="O35" s="101"/>
+      <c r="P35" s="102"/>
     </row>
     <row r="36" spans="1:22" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="13"/>
-      <c r="B36" s="75" t="s">
+      <c r="B36" s="103" t="s">
         <v>138</v>
       </c>
-      <c r="C36" s="75"/>
-      <c r="D36" s="75"/>
-      <c r="E36" s="75"/>
-      <c r="F36" s="75"/>
-      <c r="G36" s="75"/>
+      <c r="C36" s="103"/>
+      <c r="D36" s="103"/>
+      <c r="E36" s="103"/>
+      <c r="F36" s="103"/>
+      <c r="G36" s="103"/>
       <c r="H36" s="67"/>
       <c r="I36" s="13"/>
-      <c r="J36" s="75" t="s">
+      <c r="J36" s="103" t="s">
         <v>140</v>
       </c>
-      <c r="K36" s="75"/>
-      <c r="L36" s="75"/>
-      <c r="M36" s="75"/>
-      <c r="N36" s="75"/>
-      <c r="O36" s="75"/>
+      <c r="K36" s="103"/>
+      <c r="L36" s="103"/>
+      <c r="M36" s="103"/>
+      <c r="N36" s="103"/>
+      <c r="O36" s="103"/>
       <c r="P36" s="12"/>
     </row>
     <row r="37" spans="1:22" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="73" t="s">
+      <c r="A37" s="100" t="s">
         <v>81</v>
       </c>
-      <c r="B37" s="74"/>
-      <c r="C37" s="74"/>
-      <c r="D37" s="74"/>
-      <c r="E37" s="74"/>
-      <c r="F37" s="74"/>
-      <c r="G37" s="74"/>
+      <c r="B37" s="101"/>
+      <c r="C37" s="101"/>
+      <c r="D37" s="101"/>
+      <c r="E37" s="101"/>
+      <c r="F37" s="101"/>
+      <c r="G37" s="101"/>
       <c r="H37" s="66"/>
-      <c r="I37" s="73" t="s">
+      <c r="I37" s="100" t="s">
         <v>33</v>
       </c>
-      <c r="J37" s="74"/>
-      <c r="K37" s="74"/>
-      <c r="L37" s="74"/>
-      <c r="M37" s="74"/>
-      <c r="N37" s="74"/>
-      <c r="O37" s="74"/>
-      <c r="P37" s="76"/>
+      <c r="J37" s="101"/>
+      <c r="K37" s="101"/>
+      <c r="L37" s="101"/>
+      <c r="M37" s="101"/>
+      <c r="N37" s="101"/>
+      <c r="O37" s="101"/>
+      <c r="P37" s="102"/>
       <c r="S37" s="27"/>
-      <c r="T37" s="143"/>
-      <c r="U37" s="143"/>
-      <c r="V37" s="143"/>
+      <c r="T37" s="127"/>
+      <c r="U37" s="127"/>
+      <c r="V37" s="127"/>
     </row>
     <row r="38" spans="1:22" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="13"/>
-      <c r="B38" s="75" t="s">
+      <c r="B38" s="103" t="s">
         <v>134</v>
       </c>
-      <c r="C38" s="75"/>
-      <c r="D38" s="75"/>
-      <c r="E38" s="75"/>
-      <c r="F38" s="75"/>
-      <c r="G38" s="75"/>
+      <c r="C38" s="103"/>
+      <c r="D38" s="103"/>
+      <c r="E38" s="103"/>
+      <c r="F38" s="103"/>
+      <c r="G38" s="103"/>
       <c r="H38" s="67"/>
       <c r="I38" s="13"/>
-      <c r="J38" s="75" t="s">
+      <c r="J38" s="103" t="s">
         <v>134</v>
       </c>
-      <c r="K38" s="75"/>
-      <c r="L38" s="75"/>
-      <c r="M38" s="75"/>
-      <c r="N38" s="75"/>
-      <c r="O38" s="75"/>
+      <c r="K38" s="103"/>
+      <c r="L38" s="103"/>
+      <c r="M38" s="103"/>
+      <c r="N38" s="103"/>
+      <c r="O38" s="103"/>
       <c r="P38" s="12"/>
       <c r="S38" s="27"/>
       <c r="T38" s="27"/>
@@ -4397,149 +4397,149 @@
       <c r="V38" s="27"/>
     </row>
     <row r="39" spans="1:22" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="73" t="s">
+      <c r="A39" s="100" t="s">
         <v>34</v>
       </c>
-      <c r="B39" s="74"/>
-      <c r="C39" s="74"/>
-      <c r="D39" s="74"/>
-      <c r="E39" s="74"/>
-      <c r="F39" s="74"/>
-      <c r="G39" s="74"/>
+      <c r="B39" s="101"/>
+      <c r="C39" s="101"/>
+      <c r="D39" s="101"/>
+      <c r="E39" s="101"/>
+      <c r="F39" s="101"/>
+      <c r="G39" s="101"/>
       <c r="H39" s="66"/>
-      <c r="I39" s="73" t="s">
+      <c r="I39" s="100" t="s">
         <v>34</v>
       </c>
-      <c r="J39" s="74"/>
-      <c r="K39" s="74"/>
-      <c r="L39" s="74"/>
-      <c r="M39" s="74"/>
-      <c r="N39" s="74"/>
-      <c r="O39" s="74"/>
-      <c r="P39" s="76"/>
+      <c r="J39" s="101"/>
+      <c r="K39" s="101"/>
+      <c r="L39" s="101"/>
+      <c r="M39" s="101"/>
+      <c r="N39" s="101"/>
+      <c r="O39" s="101"/>
+      <c r="P39" s="102"/>
     </row>
     <row r="40" spans="1:22" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="13"/>
-      <c r="B40" s="75" t="str">
+      <c r="B40" s="103" t="str">
         <f>+VLOOKUP(B38,Hoja2!$E$2:$F$14,2,0)</f>
         <v>NJS2</v>
       </c>
-      <c r="C40" s="75"/>
-      <c r="D40" s="75"/>
-      <c r="E40" s="75"/>
-      <c r="F40" s="75"/>
-      <c r="G40" s="75"/>
+      <c r="C40" s="103"/>
+      <c r="D40" s="103"/>
+      <c r="E40" s="103"/>
+      <c r="F40" s="103"/>
+      <c r="G40" s="103"/>
       <c r="H40" s="67"/>
       <c r="I40" s="13"/>
-      <c r="J40" s="75" t="str">
+      <c r="J40" s="103" t="str">
         <f>+VLOOKUP(J38,Hoja2!$E$2:$F$14,2,0)</f>
         <v>NJS2</v>
       </c>
-      <c r="K40" s="75"/>
-      <c r="L40" s="75"/>
-      <c r="M40" s="75"/>
-      <c r="N40" s="75"/>
-      <c r="O40" s="75"/>
+      <c r="K40" s="103"/>
+      <c r="L40" s="103"/>
+      <c r="M40" s="103"/>
+      <c r="N40" s="103"/>
+      <c r="O40" s="103"/>
       <c r="P40" s="12"/>
       <c r="T40" s="29"/>
     </row>
     <row r="41" spans="1:22" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="73" t="s">
+      <c r="A41" s="100" t="s">
         <v>83</v>
       </c>
-      <c r="B41" s="74"/>
-      <c r="C41" s="74"/>
-      <c r="D41" s="74"/>
-      <c r="E41" s="74"/>
-      <c r="F41" s="74"/>
-      <c r="G41" s="74"/>
+      <c r="B41" s="101"/>
+      <c r="C41" s="101"/>
+      <c r="D41" s="101"/>
+      <c r="E41" s="101"/>
+      <c r="F41" s="101"/>
+      <c r="G41" s="101"/>
       <c r="H41" s="66"/>
-      <c r="I41" s="73" t="s">
+      <c r="I41" s="100" t="s">
         <v>32</v>
       </c>
-      <c r="J41" s="74"/>
-      <c r="K41" s="74"/>
-      <c r="L41" s="74"/>
-      <c r="M41" s="74"/>
-      <c r="N41" s="74"/>
-      <c r="O41" s="74"/>
-      <c r="P41" s="76"/>
-      <c r="T41" s="123"/>
-      <c r="U41" s="123"/>
-      <c r="V41" s="123"/>
+      <c r="J41" s="101"/>
+      <c r="K41" s="101"/>
+      <c r="L41" s="101"/>
+      <c r="M41" s="101"/>
+      <c r="N41" s="101"/>
+      <c r="O41" s="101"/>
+      <c r="P41" s="102"/>
+      <c r="T41" s="119"/>
+      <c r="U41" s="119"/>
+      <c r="V41" s="119"/>
     </row>
     <row r="42" spans="1:22" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="13"/>
-      <c r="B42" s="142">
+      <c r="B42" s="112">
         <f>+VLOOKUP(B38,Hoja2!$E$1:$G$14,3,0)</f>
         <v>2368</v>
       </c>
-      <c r="C42" s="75"/>
-      <c r="D42" s="75"/>
-      <c r="E42" s="75"/>
-      <c r="F42" s="75"/>
-      <c r="G42" s="75"/>
+      <c r="C42" s="103"/>
+      <c r="D42" s="103"/>
+      <c r="E42" s="103"/>
+      <c r="F42" s="103"/>
+      <c r="G42" s="103"/>
       <c r="H42" s="67"/>
       <c r="I42" s="13"/>
-      <c r="J42" s="142">
+      <c r="J42" s="112">
         <f>+VLOOKUP(J38,Hoja2!$E$1:$G$14,3,0)</f>
         <v>2368</v>
       </c>
-      <c r="K42" s="75"/>
-      <c r="L42" s="75"/>
-      <c r="M42" s="75"/>
-      <c r="N42" s="75"/>
-      <c r="O42" s="75"/>
+      <c r="K42" s="103"/>
+      <c r="L42" s="103"/>
+      <c r="M42" s="103"/>
+      <c r="N42" s="103"/>
+      <c r="O42" s="103"/>
       <c r="P42" s="12"/>
-      <c r="T42" s="123"/>
-      <c r="U42" s="123"/>
-      <c r="V42" s="123"/>
+      <c r="T42" s="119"/>
+      <c r="U42" s="119"/>
+      <c r="V42" s="119"/>
     </row>
     <row r="43" spans="1:22" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="73" t="s">
+      <c r="A43" s="100" t="s">
         <v>58</v>
       </c>
-      <c r="B43" s="74"/>
-      <c r="C43" s="74"/>
-      <c r="D43" s="74"/>
-      <c r="E43" s="74"/>
-      <c r="F43" s="74"/>
-      <c r="G43" s="74"/>
+      <c r="B43" s="101"/>
+      <c r="C43" s="101"/>
+      <c r="D43" s="101"/>
+      <c r="E43" s="101"/>
+      <c r="F43" s="101"/>
+      <c r="G43" s="101"/>
       <c r="H43" s="66"/>
-      <c r="I43" s="73" t="s">
+      <c r="I43" s="100" t="s">
         <v>58</v>
       </c>
-      <c r="J43" s="74"/>
-      <c r="K43" s="74"/>
-      <c r="L43" s="74"/>
-      <c r="M43" s="74"/>
-      <c r="N43" s="74"/>
-      <c r="O43" s="74"/>
-      <c r="P43" s="76"/>
+      <c r="J43" s="101"/>
+      <c r="K43" s="101"/>
+      <c r="L43" s="101"/>
+      <c r="M43" s="101"/>
+      <c r="N43" s="101"/>
+      <c r="O43" s="101"/>
+      <c r="P43" s="102"/>
     </row>
     <row r="44" spans="1:22" s="28" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13"/>
-      <c r="B44" s="133" t="s">
+      <c r="B44" s="121" t="s">
         <v>139</v>
       </c>
-      <c r="C44" s="75"/>
-      <c r="D44" s="75"/>
-      <c r="E44" s="75"/>
-      <c r="F44" s="75"/>
-      <c r="G44" s="75"/>
+      <c r="C44" s="103"/>
+      <c r="D44" s="103"/>
+      <c r="E44" s="103"/>
+      <c r="F44" s="103"/>
+      <c r="G44" s="103"/>
       <c r="H44" s="43"/>
       <c r="I44" s="13"/>
-      <c r="J44" s="133" t="s">
+      <c r="J44" s="121" t="s">
         <v>141</v>
       </c>
-      <c r="K44" s="75"/>
-      <c r="L44" s="75"/>
-      <c r="M44" s="75"/>
-      <c r="N44" s="75"/>
-      <c r="O44" s="75"/>
+      <c r="K44" s="103"/>
+      <c r="L44" s="103"/>
+      <c r="M44" s="103"/>
+      <c r="N44" s="103"/>
+      <c r="O44" s="103"/>
       <c r="P44" s="12"/>
     </row>
-    <row r="45" spans="1:22" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:22" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="10"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -4558,26 +4558,26 @@
       <c r="P45" s="3"/>
     </row>
     <row r="46" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="139" t="s">
+      <c r="A46" s="116" t="s">
         <v>65</v>
       </c>
-      <c r="B46" s="140"/>
-      <c r="C46" s="140"/>
-      <c r="D46" s="140"/>
-      <c r="E46" s="140"/>
-      <c r="F46" s="140"/>
-      <c r="G46" s="140"/>
-      <c r="H46" s="140"/>
-      <c r="I46" s="140"/>
-      <c r="J46" s="140"/>
-      <c r="K46" s="140"/>
-      <c r="L46" s="140"/>
-      <c r="M46" s="140"/>
-      <c r="N46" s="140"/>
-      <c r="O46" s="140"/>
-      <c r="P46" s="141"/>
-    </row>
-    <row r="47" spans="1:22" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="117"/>
+      <c r="C46" s="117"/>
+      <c r="D46" s="117"/>
+      <c r="E46" s="117"/>
+      <c r="F46" s="117"/>
+      <c r="G46" s="117"/>
+      <c r="H46" s="117"/>
+      <c r="I46" s="117"/>
+      <c r="J46" s="117"/>
+      <c r="K46" s="117"/>
+      <c r="L46" s="117"/>
+      <c r="M46" s="117"/>
+      <c r="N46" s="117"/>
+      <c r="O46" s="117"/>
+      <c r="P46" s="118"/>
+    </row>
+    <row r="47" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
@@ -4595,55 +4595,55 @@
       <c r="O47" s="8"/>
       <c r="P47" s="9"/>
     </row>
-    <row r="48" spans="1:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:22" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="6"/>
       <c r="B48" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C48" s="69"/>
-      <c r="D48" s="69"/>
-      <c r="E48" s="69"/>
-      <c r="F48" s="69"/>
-      <c r="G48" s="69"/>
+      <c r="C48" s="98"/>
+      <c r="D48" s="98"/>
+      <c r="E48" s="98"/>
+      <c r="F48" s="98"/>
+      <c r="G48" s="98"/>
       <c r="H48" s="1"/>
-      <c r="I48" s="77" t="s">
+      <c r="I48" s="124" t="s">
         <v>43</v>
       </c>
-      <c r="J48" s="77"/>
-      <c r="K48" s="77"/>
-      <c r="L48" s="77"/>
-      <c r="M48" s="77"/>
-      <c r="N48" s="69"/>
-      <c r="O48" s="69"/>
+      <c r="J48" s="124"/>
+      <c r="K48" s="124"/>
+      <c r="L48" s="124"/>
+      <c r="M48" s="124"/>
+      <c r="N48" s="98"/>
+      <c r="O48" s="98"/>
       <c r="P48" s="2"/>
     </row>
-    <row r="49" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="6"/>
-      <c r="B49" s="125" t="s">
+      <c r="B49" s="108" t="s">
         <v>61</v>
       </c>
-      <c r="C49" s="125"/>
-      <c r="D49" s="125"/>
-      <c r="E49" s="125"/>
-      <c r="F49" s="125"/>
-      <c r="G49" s="125"/>
+      <c r="C49" s="108"/>
+      <c r="D49" s="108"/>
+      <c r="E49" s="108"/>
+      <c r="F49" s="108"/>
+      <c r="G49" s="108"/>
       <c r="P49" s="2"/>
     </row>
-    <row r="50" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6"/>
       <c r="B50" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="C50" s="69"/>
-      <c r="D50" s="69"/>
+      <c r="C50" s="98"/>
+      <c r="D50" s="98"/>
       <c r="E50" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="F50" s="151"/>
-      <c r="G50" s="151"/>
+      <c r="F50" s="111"/>
+      <c r="G50" s="111"/>
       <c r="P50" s="2"/>
     </row>
-    <row r="51" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="6"/>
       <c r="B51" s="25"/>
       <c r="C51" s="1"/>
@@ -4655,113 +4655,113 @@
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="6"/>
-      <c r="B52" s="148" t="s">
+      <c r="B52" s="107" t="s">
         <v>64</v>
       </c>
-      <c r="C52" s="148"/>
-      <c r="D52" s="148"/>
-      <c r="E52" s="148"/>
-      <c r="F52" s="148"/>
-      <c r="G52" s="148"/>
+      <c r="C52" s="107"/>
+      <c r="D52" s="107"/>
+      <c r="E52" s="107"/>
+      <c r="F52" s="107"/>
+      <c r="G52" s="107"/>
       <c r="H52" s="26"/>
       <c r="I52" s="1"/>
       <c r="J52" s="1"/>
       <c r="K52" s="1"/>
       <c r="P52" s="2"/>
     </row>
-    <row r="53" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:16" ht="62.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="6"/>
-      <c r="B53" s="69"/>
-      <c r="C53" s="69"/>
-      <c r="D53" s="69"/>
-      <c r="F53" s="151"/>
-      <c r="G53" s="151"/>
+      <c r="B53" s="98"/>
+      <c r="C53" s="98"/>
+      <c r="D53" s="98"/>
+      <c r="F53" s="111"/>
+      <c r="G53" s="111"/>
       <c r="H53" s="26"/>
       <c r="I53" s="1"/>
       <c r="J53" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="K53" s="129"/>
-      <c r="L53" s="129"/>
-      <c r="M53" s="129"/>
-      <c r="N53" s="129"/>
+      <c r="K53" s="122"/>
+      <c r="L53" s="122"/>
+      <c r="M53" s="122"/>
+      <c r="N53" s="122"/>
       <c r="P53" s="2"/>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="6"/>
-      <c r="B54" s="147" t="s">
+      <c r="B54" s="106" t="s">
         <v>62</v>
       </c>
-      <c r="C54" s="147"/>
-      <c r="D54" s="147"/>
-      <c r="F54" s="147" t="s">
+      <c r="C54" s="106"/>
+      <c r="D54" s="106"/>
+      <c r="F54" s="106" t="s">
         <v>63</v>
       </c>
-      <c r="G54" s="147"/>
+      <c r="G54" s="106"/>
       <c r="J54" s="1"/>
-      <c r="K54" s="134" t="s">
+      <c r="K54" s="123" t="s">
         <v>35</v>
       </c>
-      <c r="L54" s="134"/>
-      <c r="M54" s="134"/>
-      <c r="N54" s="134"/>
+      <c r="L54" s="123"/>
+      <c r="M54" s="123"/>
+      <c r="N54" s="123"/>
       <c r="O54" s="40"/>
       <c r="P54" s="2"/>
     </row>
     <row r="55" spans="1:16" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="10"/>
-      <c r="G55" s="77"/>
-      <c r="H55" s="77"/>
-      <c r="I55" s="77"/>
-      <c r="J55" s="77"/>
-      <c r="K55" s="77"/>
+      <c r="G55" s="124"/>
+      <c r="H55" s="124"/>
+      <c r="I55" s="124"/>
+      <c r="J55" s="124"/>
+      <c r="K55" s="124"/>
       <c r="L55" s="1"/>
-      <c r="M55" s="77"/>
-      <c r="N55" s="77"/>
-      <c r="O55" s="77"/>
+      <c r="M55" s="124"/>
+      <c r="N55" s="124"/>
+      <c r="O55" s="124"/>
       <c r="P55" s="3"/>
     </row>
     <row r="56" spans="1:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="115" t="s">
+      <c r="A56" s="92" t="s">
         <v>60</v>
       </c>
-      <c r="B56" s="116"/>
-      <c r="C56" s="116"/>
-      <c r="D56" s="116"/>
-      <c r="E56" s="116"/>
-      <c r="F56" s="116"/>
-      <c r="G56" s="116"/>
-      <c r="H56" s="116"/>
-      <c r="I56" s="116"/>
-      <c r="J56" s="116"/>
-      <c r="K56" s="116"/>
-      <c r="L56" s="116"/>
-      <c r="M56" s="116"/>
-      <c r="N56" s="116"/>
-      <c r="O56" s="116"/>
-      <c r="P56" s="91"/>
+      <c r="B56" s="93"/>
+      <c r="C56" s="93"/>
+      <c r="D56" s="93"/>
+      <c r="E56" s="93"/>
+      <c r="F56" s="93"/>
+      <c r="G56" s="93"/>
+      <c r="H56" s="93"/>
+      <c r="I56" s="93"/>
+      <c r="J56" s="93"/>
+      <c r="K56" s="93"/>
+      <c r="L56" s="93"/>
+      <c r="M56" s="93"/>
+      <c r="N56" s="93"/>
+      <c r="O56" s="93"/>
+      <c r="P56" s="94"/>
     </row>
     <row r="57" spans="1:16" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="115" t="s">
+      <c r="A57" s="92" t="s">
         <v>59</v>
       </c>
-      <c r="B57" s="116"/>
-      <c r="C57" s="116"/>
-      <c r="D57" s="116"/>
-      <c r="E57" s="116"/>
-      <c r="F57" s="116"/>
-      <c r="G57" s="116"/>
-      <c r="H57" s="91"/>
-      <c r="I57" s="144" t="s">
+      <c r="B57" s="93"/>
+      <c r="C57" s="93"/>
+      <c r="D57" s="93"/>
+      <c r="E57" s="93"/>
+      <c r="F57" s="93"/>
+      <c r="G57" s="93"/>
+      <c r="H57" s="94"/>
+      <c r="I57" s="128" t="s">
         <v>142</v>
       </c>
-      <c r="J57" s="116"/>
-      <c r="K57" s="116"/>
-      <c r="L57" s="116"/>
-      <c r="M57" s="116"/>
-      <c r="N57" s="116"/>
-      <c r="O57" s="116"/>
-      <c r="P57" s="91"/>
+      <c r="J57" s="93"/>
+      <c r="K57" s="93"/>
+      <c r="L57" s="93"/>
+      <c r="M57" s="93"/>
+      <c r="N57" s="93"/>
+      <c r="O57" s="93"/>
+      <c r="P57" s="94"/>
     </row>
     <row r="58" spans="1:16" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="6"/>
@@ -4774,69 +4774,69 @@
       <c r="P59" s="2"/>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A60" s="135" t="s">
+      <c r="A60" s="81" t="s">
         <v>38</v>
       </c>
-      <c r="B60" s="136"/>
-      <c r="C60" s="69"/>
-      <c r="D60" s="69"/>
-      <c r="E60" s="69"/>
-      <c r="F60" s="69"/>
-      <c r="G60" s="69"/>
-      <c r="I60" s="135" t="s">
+      <c r="B60" s="82"/>
+      <c r="C60" s="98"/>
+      <c r="D60" s="98"/>
+      <c r="E60" s="98"/>
+      <c r="F60" s="98"/>
+      <c r="G60" s="98"/>
+      <c r="I60" s="81" t="s">
         <v>38</v>
       </c>
-      <c r="J60" s="136"/>
-      <c r="K60" s="69"/>
-      <c r="L60" s="69"/>
-      <c r="M60" s="69"/>
-      <c r="N60" s="69"/>
-      <c r="O60" s="69"/>
+      <c r="J60" s="82"/>
+      <c r="K60" s="98"/>
+      <c r="L60" s="98"/>
+      <c r="M60" s="98"/>
+      <c r="N60" s="98"/>
+      <c r="O60" s="98"/>
       <c r="P60" s="2"/>
     </row>
     <row r="61" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="135" t="s">
+      <c r="A61" s="81" t="s">
         <v>40</v>
       </c>
-      <c r="B61" s="136"/>
-      <c r="C61" s="155"/>
-      <c r="D61" s="155"/>
-      <c r="E61" s="155"/>
-      <c r="F61" s="155"/>
-      <c r="G61" s="155"/>
-      <c r="I61" s="135" t="s">
+      <c r="B61" s="82"/>
+      <c r="C61" s="83"/>
+      <c r="D61" s="83"/>
+      <c r="E61" s="83"/>
+      <c r="F61" s="83"/>
+      <c r="G61" s="83"/>
+      <c r="I61" s="81" t="s">
         <v>40</v>
       </c>
-      <c r="J61" s="136"/>
-      <c r="K61" s="175"/>
-      <c r="L61" s="175"/>
-      <c r="M61" s="175"/>
-      <c r="N61" s="175"/>
-      <c r="O61" s="175"/>
+      <c r="J61" s="82"/>
+      <c r="K61" s="99"/>
+      <c r="L61" s="99"/>
+      <c r="M61" s="99"/>
+      <c r="N61" s="99"/>
+      <c r="O61" s="99"/>
       <c r="P61" s="2"/>
     </row>
     <row r="62" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="135" t="s">
+      <c r="A62" s="81" t="s">
         <v>41</v>
       </c>
-      <c r="B62" s="136"/>
-      <c r="C62" s="155"/>
-      <c r="D62" s="155"/>
-      <c r="E62" s="155"/>
-      <c r="F62" s="155"/>
-      <c r="G62" s="155"/>
-      <c r="I62" s="135" t="s">
+      <c r="B62" s="82"/>
+      <c r="C62" s="83"/>
+      <c r="D62" s="83"/>
+      <c r="E62" s="83"/>
+      <c r="F62" s="83"/>
+      <c r="G62" s="83"/>
+      <c r="I62" s="81" t="s">
         <v>41</v>
       </c>
-      <c r="J62" s="136"/>
-      <c r="K62" s="176"/>
-      <c r="L62" s="176"/>
-      <c r="M62" s="176"/>
-      <c r="N62" s="176"/>
-      <c r="O62" s="176"/>
+      <c r="J62" s="82"/>
+      <c r="K62" s="97"/>
+      <c r="L62" s="97"/>
+      <c r="M62" s="97"/>
+      <c r="N62" s="97"/>
+      <c r="O62" s="97"/>
       <c r="P62" s="2"/>
     </row>
-    <row r="63" spans="1:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="10"/>
       <c r="B63" s="11"/>
       <c r="C63" s="11"/>
@@ -4861,23 +4861,23 @@
       <c r="O64" s="1"/>
     </row>
     <row r="65" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A65" s="124" t="s">
+      <c r="A65" s="120" t="s">
         <v>70</v>
       </c>
-      <c r="B65" s="124"/>
-      <c r="C65" s="124"/>
-      <c r="D65" s="124"/>
-      <c r="E65" s="124"/>
-      <c r="F65" s="124"/>
-      <c r="G65" s="124"/>
-      <c r="H65" s="124"/>
-      <c r="I65" s="124"/>
-      <c r="J65" s="124"/>
-      <c r="K65" s="124"/>
-      <c r="L65" s="124"/>
-      <c r="M65" s="124"/>
-      <c r="N65" s="124"/>
-      <c r="O65" s="124"/>
+      <c r="B65" s="120"/>
+      <c r="C65" s="120"/>
+      <c r="D65" s="120"/>
+      <c r="E65" s="120"/>
+      <c r="F65" s="120"/>
+      <c r="G65" s="120"/>
+      <c r="H65" s="120"/>
+      <c r="I65" s="120"/>
+      <c r="J65" s="120"/>
+      <c r="K65" s="120"/>
+      <c r="L65" s="120"/>
+      <c r="M65" s="120"/>
+      <c r="N65" s="120"/>
+      <c r="O65" s="120"/>
     </row>
     <row r="66" spans="1:18" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="35"/>
@@ -4897,24 +4897,24 @@
       <c r="O66" s="35"/>
     </row>
     <row r="67" spans="1:18" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="115" t="s">
+      <c r="A67" s="92" t="s">
         <v>66</v>
       </c>
-      <c r="B67" s="116"/>
-      <c r="C67" s="116"/>
-      <c r="D67" s="116"/>
-      <c r="E67" s="116"/>
-      <c r="F67" s="116"/>
-      <c r="G67" s="116"/>
-      <c r="H67" s="116"/>
-      <c r="I67" s="116"/>
-      <c r="J67" s="116"/>
-      <c r="K67" s="116"/>
-      <c r="L67" s="116"/>
-      <c r="M67" s="116"/>
-      <c r="N67" s="116"/>
-      <c r="O67" s="116"/>
-      <c r="P67" s="91"/>
+      <c r="B67" s="93"/>
+      <c r="C67" s="93"/>
+      <c r="D67" s="93"/>
+      <c r="E67" s="93"/>
+      <c r="F67" s="93"/>
+      <c r="G67" s="93"/>
+      <c r="H67" s="93"/>
+      <c r="I67" s="93"/>
+      <c r="J67" s="93"/>
+      <c r="K67" s="93"/>
+      <c r="L67" s="93"/>
+      <c r="M67" s="93"/>
+      <c r="N67" s="93"/>
+      <c r="O67" s="93"/>
+      <c r="P67" s="94"/>
     </row>
     <row r="68" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
@@ -4934,26 +4934,26 @@
       <c r="O68" s="35"/>
     </row>
     <row r="69" spans="1:18" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="158" t="s">
+      <c r="A69" s="89" t="s">
         <v>53</v>
       </c>
-      <c r="B69" s="159"/>
-      <c r="C69" s="159"/>
-      <c r="D69" s="159"/>
-      <c r="E69" s="159"/>
-      <c r="F69" s="159"/>
-      <c r="G69" s="159"/>
-      <c r="H69" s="160"/>
-      <c r="I69" s="115" t="s">
+      <c r="B69" s="90"/>
+      <c r="C69" s="90"/>
+      <c r="D69" s="90"/>
+      <c r="E69" s="90"/>
+      <c r="F69" s="90"/>
+      <c r="G69" s="90"/>
+      <c r="H69" s="91"/>
+      <c r="I69" s="92" t="s">
         <v>16</v>
       </c>
-      <c r="J69" s="116"/>
-      <c r="K69" s="116"/>
-      <c r="L69" s="116"/>
-      <c r="M69" s="116"/>
-      <c r="N69" s="116"/>
-      <c r="O69" s="116"/>
-      <c r="P69" s="91"/>
+      <c r="J69" s="93"/>
+      <c r="K69" s="93"/>
+      <c r="L69" s="93"/>
+      <c r="M69" s="93"/>
+      <c r="N69" s="93"/>
+      <c r="O69" s="93"/>
+      <c r="P69" s="94"/>
     </row>
     <row r="70" spans="1:18" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="20"/>
@@ -5036,14 +5036,14 @@
       <c r="B74" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="C74" s="127" t="str">
+      <c r="C74" s="95" t="str">
         <f>+A6&amp;" "&amp;I6</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="D74" s="127"/>
-      <c r="E74" s="127"/>
-      <c r="F74" s="127"/>
-      <c r="G74" s="127"/>
+      <c r="D74" s="95"/>
+      <c r="E74" s="95"/>
+      <c r="F74" s="95"/>
+      <c r="G74" s="95"/>
       <c r="H74" s="37"/>
       <c r="I74" s="6"/>
       <c r="J74" s="25" t="s">
@@ -5061,14 +5061,14 @@
       <c r="B75" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="C75" s="161">
+      <c r="C75" s="96">
         <f>+K5</f>
         <v>46121</v>
       </c>
-      <c r="D75" s="127"/>
-      <c r="E75" s="127"/>
-      <c r="F75" s="127"/>
-      <c r="G75" s="127"/>
+      <c r="D75" s="95"/>
+      <c r="E75" s="95"/>
+      <c r="F75" s="95"/>
+      <c r="G75" s="95"/>
       <c r="H75" s="37"/>
       <c r="I75" s="6"/>
       <c r="J75" s="25" t="s">
@@ -5094,13 +5094,13 @@
       <c r="G76" s="57"/>
       <c r="H76" s="37"/>
       <c r="I76" s="6"/>
-      <c r="K76" s="156" t="s">
+      <c r="K76" s="87" t="s">
         <v>69</v>
       </c>
-      <c r="L76" s="156"/>
-      <c r="M76" s="156"/>
-      <c r="N76" s="156"/>
-      <c r="O76" s="156"/>
+      <c r="L76" s="87"/>
+      <c r="M76" s="87"/>
+      <c r="N76" s="87"/>
+      <c r="O76" s="87"/>
       <c r="P76" s="2"/>
       <c r="R76" s="56" t="s">
         <v>68</v>
@@ -5113,11 +5113,11 @@
       <c r="J77" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="K77" s="157"/>
-      <c r="L77" s="157"/>
-      <c r="M77" s="157"/>
-      <c r="N77" s="157"/>
-      <c r="O77" s="157"/>
+      <c r="K77" s="88"/>
+      <c r="L77" s="88"/>
+      <c r="M77" s="88"/>
+      <c r="N77" s="88"/>
+      <c r="O77" s="88"/>
       <c r="P77" s="2"/>
       <c r="R77" s="56" t="s">
         <v>68</v>
@@ -5128,11 +5128,11 @@
       <c r="H78" s="2"/>
       <c r="I78" s="6"/>
       <c r="J78" s="25"/>
-      <c r="K78" s="157"/>
-      <c r="L78" s="157"/>
-      <c r="M78" s="157"/>
-      <c r="N78" s="157"/>
-      <c r="O78" s="157"/>
+      <c r="K78" s="88"/>
+      <c r="L78" s="88"/>
+      <c r="M78" s="88"/>
+      <c r="N78" s="88"/>
+      <c r="O78" s="88"/>
       <c r="P78" s="2"/>
       <c r="R78" s="56"/>
     </row>
@@ -5140,11 +5140,11 @@
       <c r="A79" s="13"/>
       <c r="H79" s="2"/>
       <c r="I79" s="6"/>
-      <c r="K79" s="157"/>
-      <c r="L79" s="157"/>
-      <c r="M79" s="157"/>
-      <c r="N79" s="157"/>
-      <c r="O79" s="157"/>
+      <c r="K79" s="88"/>
+      <c r="L79" s="88"/>
+      <c r="M79" s="88"/>
+      <c r="N79" s="88"/>
+      <c r="O79" s="88"/>
       <c r="P79" s="2"/>
     </row>
     <row r="80" spans="1:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -5183,28 +5183,28 @@
       <c r="O81" s="30"/>
     </row>
     <row r="82" spans="1:22" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="92" t="s">
+      <c r="A82" s="129" t="s">
         <v>50</v>
       </c>
-      <c r="B82" s="92"/>
-      <c r="C82" s="92"/>
-      <c r="D82" s="92"/>
-      <c r="E82" s="92"/>
-      <c r="F82" s="92" t="s">
+      <c r="B82" s="129"/>
+      <c r="C82" s="129"/>
+      <c r="D82" s="129"/>
+      <c r="E82" s="129"/>
+      <c r="F82" s="129" t="s">
         <v>51</v>
       </c>
-      <c r="G82" s="92"/>
-      <c r="H82" s="92"/>
-      <c r="I82" s="92"/>
-      <c r="J82" s="92"/>
-      <c r="K82" s="92"/>
-      <c r="L82" s="92" t="s">
+      <c r="G82" s="129"/>
+      <c r="H82" s="129"/>
+      <c r="I82" s="129"/>
+      <c r="J82" s="129"/>
+      <c r="K82" s="129"/>
+      <c r="L82" s="129" t="s">
         <v>52</v>
       </c>
-      <c r="M82" s="92"/>
-      <c r="N82" s="92"/>
-      <c r="O82" s="92"/>
-      <c r="P82" s="92"/>
+      <c r="M82" s="129"/>
+      <c r="N82" s="129"/>
+      <c r="O82" s="129"/>
+      <c r="P82" s="129"/>
     </row>
     <row r="83" spans="1:22" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="14"/>
@@ -5273,23 +5273,23 @@
       <c r="B86" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C86" s="162"/>
-      <c r="D86" s="162"/>
-      <c r="E86" s="163"/>
-      <c r="F86" s="164" t="s">
+      <c r="C86" s="84"/>
+      <c r="D86" s="84"/>
+      <c r="E86" s="132"/>
+      <c r="F86" s="69" t="s">
         <v>38</v>
       </c>
-      <c r="G86" s="162"/>
-      <c r="H86" s="162"/>
-      <c r="I86" s="162"/>
-      <c r="J86" s="162"/>
-      <c r="K86" s="163"/>
-      <c r="L86" s="164" t="s">
+      <c r="G86" s="84"/>
+      <c r="H86" s="84"/>
+      <c r="I86" s="84"/>
+      <c r="J86" s="84"/>
+      <c r="K86" s="132"/>
+      <c r="L86" s="69" t="s">
         <v>38</v>
       </c>
-      <c r="M86" s="162"/>
-      <c r="N86" s="162"/>
-      <c r="O86" s="162"/>
+      <c r="M86" s="84"/>
+      <c r="N86" s="84"/>
+      <c r="O86" s="84"/>
       <c r="P86" s="2"/>
       <c r="S86" s="25"/>
       <c r="T86" s="26"/>
@@ -5301,51 +5301,51 @@
       <c r="B87" s="59" t="s">
         <v>40</v>
       </c>
-      <c r="C87" s="165"/>
-      <c r="D87" s="165"/>
-      <c r="E87" s="166"/>
-      <c r="F87" s="164" t="s">
+      <c r="C87" s="85"/>
+      <c r="D87" s="85"/>
+      <c r="E87" s="86"/>
+      <c r="F87" s="69" t="s">
         <v>40</v>
       </c>
-      <c r="G87" s="162"/>
-      <c r="H87" s="162"/>
-      <c r="I87" s="162"/>
-      <c r="J87" s="162"/>
-      <c r="K87" s="163"/>
-      <c r="L87" s="164" t="s">
+      <c r="G87" s="84"/>
+      <c r="H87" s="84"/>
+      <c r="I87" s="84"/>
+      <c r="J87" s="84"/>
+      <c r="K87" s="132"/>
+      <c r="L87" s="69" t="s">
         <v>40</v>
       </c>
-      <c r="M87" s="165"/>
-      <c r="N87" s="165"/>
-      <c r="O87" s="166"/>
+      <c r="M87" s="85"/>
+      <c r="N87" s="85"/>
+      <c r="O87" s="86"/>
       <c r="P87" s="42"/>
       <c r="S87" s="25"/>
-      <c r="T87" s="125"/>
-      <c r="U87" s="125"/>
-      <c r="V87" s="125"/>
+      <c r="T87" s="108"/>
+      <c r="U87" s="108"/>
+      <c r="V87" s="108"/>
     </row>
     <row r="88" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="6"/>
       <c r="B88" s="59" t="s">
         <v>41</v>
       </c>
-      <c r="C88" s="165"/>
-      <c r="D88" s="165"/>
-      <c r="E88" s="166"/>
-      <c r="F88" s="164" t="s">
+      <c r="C88" s="85"/>
+      <c r="D88" s="85"/>
+      <c r="E88" s="86"/>
+      <c r="F88" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="G88" s="162"/>
-      <c r="H88" s="162"/>
-      <c r="I88" s="162"/>
-      <c r="J88" s="162"/>
-      <c r="K88" s="163"/>
-      <c r="L88" s="164" t="s">
+      <c r="G88" s="84"/>
+      <c r="H88" s="84"/>
+      <c r="I88" s="84"/>
+      <c r="J88" s="84"/>
+      <c r="K88" s="132"/>
+      <c r="L88" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="M88" s="165"/>
-      <c r="N88" s="165"/>
-      <c r="O88" s="166"/>
+      <c r="M88" s="85"/>
+      <c r="N88" s="85"/>
+      <c r="O88" s="86"/>
       <c r="P88" s="37"/>
       <c r="S88" s="25"/>
       <c r="T88" s="26"/>
@@ -5355,19 +5355,19 @@
     <row r="89" spans="1:22" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="15"/>
       <c r="B89" s="17"/>
-      <c r="C89" s="167"/>
-      <c r="D89" s="167"/>
-      <c r="E89" s="168"/>
-      <c r="F89" s="169"/>
-      <c r="G89" s="170"/>
-      <c r="H89" s="170"/>
-      <c r="I89" s="171"/>
-      <c r="J89" s="167"/>
-      <c r="K89" s="172"/>
-      <c r="L89" s="173"/>
-      <c r="M89" s="174"/>
-      <c r="N89" s="174"/>
-      <c r="O89" s="174"/>
+      <c r="C89" s="70"/>
+      <c r="D89" s="70"/>
+      <c r="E89" s="71"/>
+      <c r="F89" s="72"/>
+      <c r="G89" s="73"/>
+      <c r="H89" s="73"/>
+      <c r="I89" s="74"/>
+      <c r="J89" s="70"/>
+      <c r="K89" s="75"/>
+      <c r="L89" s="76"/>
+      <c r="M89" s="77"/>
+      <c r="N89" s="77"/>
+      <c r="O89" s="77"/>
       <c r="P89" s="3"/>
     </row>
     <row r="90" spans="1:22" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -5423,24 +5423,24 @@
       <c r="O92" s="30"/>
     </row>
     <row r="93" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="131" t="s">
+      <c r="A93" s="134" t="s">
         <v>54</v>
       </c>
-      <c r="B93" s="131"/>
-      <c r="C93" s="131"/>
-      <c r="D93" s="131"/>
-      <c r="E93" s="131"/>
-      <c r="F93" s="131"/>
-      <c r="G93" s="131"/>
-      <c r="H93" s="131"/>
-      <c r="I93" s="131"/>
-      <c r="J93" s="131"/>
-      <c r="K93" s="131"/>
-      <c r="L93" s="131"/>
-      <c r="M93" s="131"/>
-      <c r="N93" s="131"/>
-      <c r="O93" s="131"/>
-      <c r="P93" s="131"/>
+      <c r="B93" s="134"/>
+      <c r="C93" s="134"/>
+      <c r="D93" s="134"/>
+      <c r="E93" s="134"/>
+      <c r="F93" s="134"/>
+      <c r="G93" s="134"/>
+      <c r="H93" s="134"/>
+      <c r="I93" s="134"/>
+      <c r="J93" s="134"/>
+      <c r="K93" s="134"/>
+      <c r="L93" s="134"/>
+      <c r="M93" s="134"/>
+      <c r="N93" s="134"/>
+      <c r="O93" s="134"/>
+      <c r="P93" s="134"/>
     </row>
     <row r="94" spans="1:22" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" s="44"/>
@@ -5479,24 +5479,24 @@
       <c r="P95" s="49"/>
     </row>
     <row r="96" spans="1:22" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="115" t="s">
+      <c r="A96" s="92" t="s">
         <v>55</v>
       </c>
-      <c r="B96" s="116"/>
-      <c r="C96" s="116"/>
-      <c r="D96" s="116"/>
-      <c r="E96" s="116"/>
-      <c r="F96" s="116"/>
-      <c r="G96" s="116"/>
-      <c r="H96" s="116"/>
-      <c r="I96" s="116"/>
-      <c r="J96" s="116"/>
-      <c r="K96" s="116"/>
-      <c r="L96" s="116"/>
-      <c r="M96" s="116"/>
-      <c r="N96" s="116"/>
-      <c r="O96" s="116"/>
-      <c r="P96" s="91"/>
+      <c r="B96" s="93"/>
+      <c r="C96" s="93"/>
+      <c r="D96" s="93"/>
+      <c r="E96" s="93"/>
+      <c r="F96" s="93"/>
+      <c r="G96" s="93"/>
+      <c r="H96" s="93"/>
+      <c r="I96" s="93"/>
+      <c r="J96" s="93"/>
+      <c r="K96" s="93"/>
+      <c r="L96" s="93"/>
+      <c r="M96" s="93"/>
+      <c r="N96" s="93"/>
+      <c r="O96" s="93"/>
+      <c r="P96" s="94"/>
     </row>
     <row r="97" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="19"/>
@@ -5573,17 +5573,17 @@
       <c r="C101" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="D101" s="128"/>
-      <c r="E101" s="129"/>
-      <c r="F101" s="129"/>
+      <c r="D101" s="131"/>
+      <c r="E101" s="122"/>
+      <c r="F101" s="122"/>
       <c r="H101" s="26"/>
       <c r="I101" s="30"/>
       <c r="J101" s="51" t="s">
         <v>44</v>
       </c>
-      <c r="K101" s="129"/>
-      <c r="L101" s="129"/>
-      <c r="M101" s="129"/>
+      <c r="K101" s="122"/>
+      <c r="L101" s="122"/>
+      <c r="M101" s="122"/>
       <c r="N101" s="1"/>
       <c r="P101" s="2"/>
     </row>
@@ -5599,9 +5599,9 @@
       <c r="C103" s="51" t="s">
         <v>46</v>
       </c>
-      <c r="D103" s="126"/>
-      <c r="E103" s="126"/>
-      <c r="F103" s="126"/>
+      <c r="D103" s="130"/>
+      <c r="E103" s="130"/>
+      <c r="F103" s="130"/>
       <c r="H103" s="26"/>
       <c r="I103" s="27"/>
       <c r="O103" s="30"/>
@@ -5611,9 +5611,9 @@
       <c r="A104" s="13"/>
       <c r="B104" s="28"/>
       <c r="C104" s="28"/>
-      <c r="D104" s="126"/>
-      <c r="E104" s="126"/>
-      <c r="F104" s="126"/>
+      <c r="D104" s="130"/>
+      <c r="E104" s="130"/>
+      <c r="F104" s="130"/>
       <c r="H104" s="26"/>
       <c r="I104" s="30"/>
       <c r="J104" s="28"/>
@@ -5624,9 +5624,9 @@
       <c r="A105" s="13"/>
       <c r="B105" s="28"/>
       <c r="C105" s="28"/>
-      <c r="D105" s="132"/>
-      <c r="E105" s="132"/>
-      <c r="F105" s="132"/>
+      <c r="D105" s="135"/>
+      <c r="E105" s="135"/>
+      <c r="F105" s="135"/>
       <c r="G105" s="26"/>
       <c r="H105" s="26"/>
       <c r="I105" s="30"/>
@@ -5656,12 +5656,12 @@
       <c r="C107" s="28"/>
       <c r="D107" s="28"/>
       <c r="E107" s="26"/>
-      <c r="F107" s="77"/>
-      <c r="G107" s="77"/>
-      <c r="H107" s="77"/>
-      <c r="I107" s="77"/>
-      <c r="J107" s="77"/>
-      <c r="K107" s="77"/>
+      <c r="F107" s="124"/>
+      <c r="G107" s="124"/>
+      <c r="H107" s="124"/>
+      <c r="I107" s="124"/>
+      <c r="J107" s="124"/>
+      <c r="K107" s="124"/>
       <c r="O107" s="30"/>
       <c r="P107" s="2"/>
     </row>
@@ -5686,14 +5686,14 @@
       <c r="C109" s="55"/>
       <c r="D109" s="55"/>
       <c r="E109" s="28"/>
-      <c r="F109" s="130" t="s">
+      <c r="F109" s="133" t="s">
         <v>67</v>
       </c>
-      <c r="G109" s="130"/>
-      <c r="H109" s="130"/>
-      <c r="I109" s="130"/>
-      <c r="J109" s="130"/>
-      <c r="K109" s="130"/>
+      <c r="G109" s="133"/>
+      <c r="H109" s="133"/>
+      <c r="I109" s="133"/>
+      <c r="J109" s="133"/>
+      <c r="K109" s="133"/>
       <c r="O109" s="30"/>
       <c r="P109" s="2"/>
     </row>
@@ -5721,11 +5721,11 @@
       <c r="F111" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="G111" s="126"/>
-      <c r="H111" s="126"/>
-      <c r="I111" s="126"/>
-      <c r="J111" s="126"/>
-      <c r="K111" s="126"/>
+      <c r="G111" s="130"/>
+      <c r="H111" s="130"/>
+      <c r="I111" s="130"/>
+      <c r="J111" s="130"/>
+      <c r="K111" s="130"/>
       <c r="O111" s="30"/>
       <c r="P111" s="2"/>
     </row>
@@ -5738,11 +5738,11 @@
       <c r="F112" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="G112" s="127"/>
-      <c r="H112" s="127"/>
-      <c r="I112" s="127"/>
-      <c r="J112" s="127"/>
-      <c r="K112" s="127"/>
+      <c r="G112" s="95"/>
+      <c r="H112" s="95"/>
+      <c r="I112" s="95"/>
+      <c r="J112" s="95"/>
+      <c r="K112" s="95"/>
       <c r="O112" s="30"/>
       <c r="P112" s="2"/>
     </row>
@@ -5760,22 +5760,22 @@
     </row>
     <row r="114" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="13"/>
-      <c r="B114" s="75" t="s">
+      <c r="B114" s="103" t="s">
         <v>37</v>
       </c>
-      <c r="C114" s="75"/>
-      <c r="D114" s="75"/>
-      <c r="E114" s="75"/>
-      <c r="F114" s="75"/>
-      <c r="G114" s="75"/>
-      <c r="H114" s="75"/>
-      <c r="I114" s="75"/>
-      <c r="J114" s="75"/>
-      <c r="K114" s="75"/>
-      <c r="L114" s="75"/>
-      <c r="M114" s="75"/>
-      <c r="N114" s="75"/>
-      <c r="O114" s="75"/>
+      <c r="C114" s="103"/>
+      <c r="D114" s="103"/>
+      <c r="E114" s="103"/>
+      <c r="F114" s="103"/>
+      <c r="G114" s="103"/>
+      <c r="H114" s="103"/>
+      <c r="I114" s="103"/>
+      <c r="J114" s="103"/>
+      <c r="K114" s="103"/>
+      <c r="L114" s="103"/>
+      <c r="M114" s="103"/>
+      <c r="N114" s="103"/>
+      <c r="O114" s="103"/>
       <c r="P114" s="2"/>
     </row>
     <row r="115" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5832,23 +5832,23 @@
       <c r="O117" s="30"/>
     </row>
     <row r="118" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A118" s="124" t="s">
+      <c r="A118" s="120" t="s">
         <v>70</v>
       </c>
-      <c r="B118" s="124"/>
-      <c r="C118" s="124"/>
-      <c r="D118" s="124"/>
-      <c r="E118" s="124"/>
-      <c r="F118" s="124"/>
-      <c r="G118" s="124"/>
-      <c r="H118" s="124"/>
-      <c r="I118" s="124"/>
-      <c r="J118" s="124"/>
-      <c r="K118" s="124"/>
-      <c r="L118" s="124"/>
-      <c r="M118" s="124"/>
-      <c r="N118" s="124"/>
-      <c r="O118" s="124"/>
+      <c r="B118" s="120"/>
+      <c r="C118" s="120"/>
+      <c r="D118" s="120"/>
+      <c r="E118" s="120"/>
+      <c r="F118" s="120"/>
+      <c r="G118" s="120"/>
+      <c r="H118" s="120"/>
+      <c r="I118" s="120"/>
+      <c r="J118" s="120"/>
+      <c r="K118" s="120"/>
+      <c r="L118" s="120"/>
+      <c r="M118" s="120"/>
+      <c r="N118" s="120"/>
+      <c r="O118" s="120"/>
     </row>
     <row r="119" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="28"/>
@@ -5869,6 +5869,126 @@
     </row>
   </sheetData>
   <mergeCells count="144">
+    <mergeCell ref="C48:G48"/>
+    <mergeCell ref="E11:H11"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="J30:O30"/>
+    <mergeCell ref="J28:O28"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="I29:P29"/>
+    <mergeCell ref="J38:O38"/>
+    <mergeCell ref="J36:O36"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="I31:P31"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="I11:L11"/>
+    <mergeCell ref="M11:P11"/>
+    <mergeCell ref="A12:P12"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="M16:O16"/>
+    <mergeCell ref="M17:O17"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="C88:E88"/>
+    <mergeCell ref="K1:P1"/>
+    <mergeCell ref="K2:P2"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K4:P4"/>
+    <mergeCell ref="K5:P5"/>
+    <mergeCell ref="A1:J5"/>
+    <mergeCell ref="E9:H10"/>
+    <mergeCell ref="I6:P7"/>
+    <mergeCell ref="I8:P8"/>
+    <mergeCell ref="I9:P9"/>
+    <mergeCell ref="A9:D10"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="M22:O22"/>
+    <mergeCell ref="I25:P25"/>
+    <mergeCell ref="I48:M48"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="M3:P3"/>
+    <mergeCell ref="A6:H7"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="M10:P10"/>
+    <mergeCell ref="I10:L10"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="T41:V41"/>
+    <mergeCell ref="A118:O118"/>
+    <mergeCell ref="T87:V87"/>
+    <mergeCell ref="A96:P96"/>
+    <mergeCell ref="L82:P82"/>
+    <mergeCell ref="F107:K107"/>
+    <mergeCell ref="B114:O114"/>
+    <mergeCell ref="G111:K111"/>
+    <mergeCell ref="G112:K112"/>
+    <mergeCell ref="A82:E82"/>
+    <mergeCell ref="F82:K82"/>
+    <mergeCell ref="D101:F101"/>
+    <mergeCell ref="K101:M101"/>
+    <mergeCell ref="M88:O88"/>
+    <mergeCell ref="G86:K86"/>
+    <mergeCell ref="G87:K87"/>
+    <mergeCell ref="G88:K88"/>
+    <mergeCell ref="F109:K109"/>
+    <mergeCell ref="A93:P93"/>
+    <mergeCell ref="D105:F105"/>
+    <mergeCell ref="D103:F103"/>
+    <mergeCell ref="D104:F104"/>
+    <mergeCell ref="C86:E86"/>
+    <mergeCell ref="C87:E87"/>
+    <mergeCell ref="T42:V42"/>
+    <mergeCell ref="A65:O65"/>
+    <mergeCell ref="B32:G32"/>
+    <mergeCell ref="B34:G34"/>
+    <mergeCell ref="I43:P43"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="J44:O44"/>
+    <mergeCell ref="B44:G44"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="K53:N53"/>
+    <mergeCell ref="K54:N54"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="M55:O55"/>
+    <mergeCell ref="G55:K55"/>
+    <mergeCell ref="A56:P56"/>
+    <mergeCell ref="N48:O48"/>
+    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="A57:H57"/>
+    <mergeCell ref="A46:P46"/>
+    <mergeCell ref="J42:O42"/>
+    <mergeCell ref="J40:O40"/>
+    <mergeCell ref="T37:V37"/>
+    <mergeCell ref="I57:P57"/>
+    <mergeCell ref="I60:J60"/>
+    <mergeCell ref="G20:O20"/>
+    <mergeCell ref="M18:O18"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="F54:G54"/>
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B49:G49"/>
+    <mergeCell ref="K60:O60"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="I41:P41"/>
+    <mergeCell ref="A24:O24"/>
+    <mergeCell ref="C50:D50"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="B40:G40"/>
+    <mergeCell ref="I37:P37"/>
+    <mergeCell ref="I39:P39"/>
+    <mergeCell ref="B42:G42"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="I27:P27"/>
+    <mergeCell ref="A23:P23"/>
+    <mergeCell ref="B18:C18"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B21:L21"/>
     <mergeCell ref="M21:O21"/>
@@ -5893,126 +6013,6 @@
     <mergeCell ref="I35:P35"/>
     <mergeCell ref="J34:O34"/>
     <mergeCell ref="J32:O32"/>
-    <mergeCell ref="I60:J60"/>
-    <mergeCell ref="G20:O20"/>
-    <mergeCell ref="M18:O18"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="F54:G54"/>
-    <mergeCell ref="B52:G52"/>
-    <mergeCell ref="B49:G49"/>
-    <mergeCell ref="K60:O60"/>
-    <mergeCell ref="A41:G41"/>
-    <mergeCell ref="I41:P41"/>
-    <mergeCell ref="A24:O24"/>
-    <mergeCell ref="C50:D50"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="B53:D53"/>
-    <mergeCell ref="A39:G39"/>
-    <mergeCell ref="B40:G40"/>
-    <mergeCell ref="I37:P37"/>
-    <mergeCell ref="I39:P39"/>
-    <mergeCell ref="B42:G42"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="I27:P27"/>
-    <mergeCell ref="A23:P23"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="T42:V42"/>
-    <mergeCell ref="A65:O65"/>
-    <mergeCell ref="B32:G32"/>
-    <mergeCell ref="B34:G34"/>
-    <mergeCell ref="I43:P43"/>
-    <mergeCell ref="A33:G33"/>
-    <mergeCell ref="J44:O44"/>
-    <mergeCell ref="B44:G44"/>
-    <mergeCell ref="A43:G43"/>
-    <mergeCell ref="K53:N53"/>
-    <mergeCell ref="K54:N54"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="M55:O55"/>
-    <mergeCell ref="G55:K55"/>
-    <mergeCell ref="A56:P56"/>
-    <mergeCell ref="N48:O48"/>
-    <mergeCell ref="A35:G35"/>
-    <mergeCell ref="B36:G36"/>
-    <mergeCell ref="A57:H57"/>
-    <mergeCell ref="A46:P46"/>
-    <mergeCell ref="J42:O42"/>
-    <mergeCell ref="J40:O40"/>
-    <mergeCell ref="T37:V37"/>
-    <mergeCell ref="I57:P57"/>
-    <mergeCell ref="T41:V41"/>
-    <mergeCell ref="A118:O118"/>
-    <mergeCell ref="T87:V87"/>
-    <mergeCell ref="A96:P96"/>
-    <mergeCell ref="L82:P82"/>
-    <mergeCell ref="F107:K107"/>
-    <mergeCell ref="B114:O114"/>
-    <mergeCell ref="G111:K111"/>
-    <mergeCell ref="G112:K112"/>
-    <mergeCell ref="A82:E82"/>
-    <mergeCell ref="F82:K82"/>
-    <mergeCell ref="D101:F101"/>
-    <mergeCell ref="K101:M101"/>
-    <mergeCell ref="M88:O88"/>
-    <mergeCell ref="G86:K86"/>
-    <mergeCell ref="G87:K87"/>
-    <mergeCell ref="G88:K88"/>
-    <mergeCell ref="F109:K109"/>
-    <mergeCell ref="A93:P93"/>
-    <mergeCell ref="D105:F105"/>
-    <mergeCell ref="D103:F103"/>
-    <mergeCell ref="D104:F104"/>
-    <mergeCell ref="C86:E86"/>
-    <mergeCell ref="C87:E87"/>
-    <mergeCell ref="C88:E88"/>
-    <mergeCell ref="K1:P1"/>
-    <mergeCell ref="K2:P2"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="K4:P4"/>
-    <mergeCell ref="K5:P5"/>
-    <mergeCell ref="A1:J5"/>
-    <mergeCell ref="E9:H10"/>
-    <mergeCell ref="I6:P7"/>
-    <mergeCell ref="I8:P8"/>
-    <mergeCell ref="I9:P9"/>
-    <mergeCell ref="A9:D10"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="M22:O22"/>
-    <mergeCell ref="I25:P25"/>
-    <mergeCell ref="I48:M48"/>
-    <mergeCell ref="A27:G27"/>
-    <mergeCell ref="M3:P3"/>
-    <mergeCell ref="A6:H7"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="M10:P10"/>
-    <mergeCell ref="I10:L10"/>
-    <mergeCell ref="B28:G28"/>
-    <mergeCell ref="B30:G30"/>
-    <mergeCell ref="C48:G48"/>
-    <mergeCell ref="E11:H11"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A29:G29"/>
-    <mergeCell ref="J30:O30"/>
-    <mergeCell ref="J28:O28"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="I29:P29"/>
-    <mergeCell ref="J38:O38"/>
-    <mergeCell ref="J36:O36"/>
-    <mergeCell ref="A37:G37"/>
-    <mergeCell ref="B38:G38"/>
-    <mergeCell ref="I31:P31"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="I11:L11"/>
-    <mergeCell ref="M11:P11"/>
-    <mergeCell ref="A12:P12"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="M15:O15"/>
-    <mergeCell ref="M16:O16"/>
-    <mergeCell ref="M17:O17"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H28" xr:uid="{10E01B42-B597-402D-BF88-0ACA852BE5A5}">
@@ -6422,7 +6422,7 @@
                     <xdr:col>10</xdr:col>
                     <xdr:colOff>742950</xdr:colOff>
                     <xdr:row>21</xdr:row>
-                    <xdr:rowOff>38100</xdr:rowOff>
+                    <xdr:rowOff>66675</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -6444,7 +6444,7 @@
                     <xdr:col>12</xdr:col>
                     <xdr:colOff>714375</xdr:colOff>
                     <xdr:row>21</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>38100</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>

</xml_diff>